<commit_message>
Removed emission lines with S/R < 3 from raw spectral data.
</commit_message>
<xml_diff>
--- a/Extra Abundances/Final_CLASSY_EMISSION_LINES_David.xlsx
+++ b/Extra Abundances/Final_CLASSY_EMISSION_LINES_David.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0013ccd3bb406478/Senior Honours Project/CLASSY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0013ccd3bb406478/Senior Honours Project/Extra Abundances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6A61F873-5642-1F4E-9EEC-E5CE1B3A1FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9015C607-DFF2-40FF-8FFB-B926460CB849}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{6A61F873-5642-1F4E-9EEC-E5CE1B3A1FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76847961-7BBE-4949-83B7-E73447612703}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{61282016-CF89-B44E-B0FA-48962238AFD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="145">
   <si>
     <t>galaxy</t>
   </si>
@@ -560,6 +560,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1598,17 +1602,17 @@
       <c r="AI3" s="1">
         <v>3.0628255336346002</v>
       </c>
-      <c r="AJ3" s="1">
-        <v>4.8757526959034798E-2</v>
-      </c>
-      <c r="AK3" s="1">
-        <v>1.65602122086848E-2</v>
-      </c>
-      <c r="AL3" s="1">
-        <v>1.6586361483355599E-2</v>
-      </c>
-      <c r="AM3" s="1">
-        <v>2.94193466041175</v>
+      <c r="AJ3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN3" s="1">
         <v>107.617599621555</v>
@@ -2166,17 +2170,17 @@
       <c r="Y5" s="1">
         <v>4.6687529309554003</v>
       </c>
-      <c r="Z5" s="1">
-        <v>0.374293915276254</v>
-      </c>
-      <c r="AA5" s="1">
-        <v>0.15546965932588599</v>
-      </c>
-      <c r="AB5" s="1">
-        <v>0.155018332234276</v>
-      </c>
-      <c r="AC5" s="1">
-        <v>2.4110114810916601</v>
+      <c r="Z5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AD5" s="1">
         <v>0.46512883249918502</v>
@@ -2184,41 +2188,41 @@
       <c r="AE5" s="1">
         <v>3.2478982696261598</v>
       </c>
-      <c r="AF5" s="1">
-        <v>0.18055306326866699</v>
-      </c>
-      <c r="AG5" s="1">
-        <v>0.14708986184477599</v>
-      </c>
-      <c r="AH5" s="1">
-        <v>0.146644285620185</v>
-      </c>
-      <c r="AI5" s="1">
-        <v>1.22936474150082</v>
-      </c>
-      <c r="AJ5" s="1">
-        <v>0.29429722531306901</v>
-      </c>
-      <c r="AK5" s="1">
-        <v>0.141445267627859</v>
-      </c>
-      <c r="AL5" s="1">
-        <v>0.14109043692641901</v>
-      </c>
-      <c r="AM5" s="1">
-        <v>2.08326140861148</v>
-      </c>
-      <c r="AN5" s="1">
-        <v>6.04629608188145</v>
-      </c>
-      <c r="AO5" s="1">
-        <v>2.2237641495198002</v>
-      </c>
-      <c r="AP5" s="1">
-        <v>2.22339606041289</v>
-      </c>
-      <c r="AQ5" s="1">
-        <v>2.7191811143859201</v>
+      <c r="AF5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AO5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AP5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AQ5" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AR5" s="1">
         <v>7.6363977544097397</v>
@@ -2268,17 +2272,17 @@
       <c r="BG5" s="1">
         <v>2.0947502149524002</v>
       </c>
-      <c r="BH5" s="4">
-        <v>0.21993948429635801</v>
-      </c>
-      <c r="BI5" s="4">
-        <v>8.3514261293355402E-2</v>
-      </c>
-      <c r="BJ5" s="4">
-        <v>8.3514261293355402E-2</v>
-      </c>
-      <c r="BK5" s="4">
-        <v>2.6391608262727302</v>
+      <c r="BH5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BI5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BJ5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BK5" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="BL5" s="1">
         <v>56.248252533843697</v>
@@ -2292,17 +2296,17 @@
       <c r="BO5" s="1">
         <v>24.542019267787701</v>
       </c>
-      <c r="BP5" s="1">
-        <v>0.453388007441202</v>
-      </c>
-      <c r="BQ5" s="1">
-        <v>0.26445205403917099</v>
-      </c>
-      <c r="BR5" s="1">
-        <v>0.26488103298764698</v>
-      </c>
-      <c r="BS5" s="1">
-        <v>1.7130548751922701</v>
+      <c r="BP5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BQ5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BR5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BS5" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="BT5" s="1">
         <v>2.4709822828741901</v>
@@ -2782,29 +2786,29 @@
       <c r="AE7" s="1">
         <v>8.1438796978036994</v>
       </c>
-      <c r="AF7" s="1">
-        <v>6.0914435194519799E-3</v>
-      </c>
-      <c r="AG7" s="1">
-        <v>4.3580032641837296E-3</v>
-      </c>
-      <c r="AH7" s="1">
-        <v>4.3424821818709098E-3</v>
-      </c>
-      <c r="AI7" s="1">
-        <v>1.4002537361815901</v>
-      </c>
-      <c r="AJ7" s="1">
-        <v>9.9385317317093307E-3</v>
-      </c>
-      <c r="AK7" s="1">
-        <v>3.5697598705212298E-3</v>
-      </c>
-      <c r="AL7" s="1">
-        <v>3.55949084975728E-3</v>
-      </c>
-      <c r="AM7" s="1">
-        <v>2.7881001247516299</v>
+      <c r="AF7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM7" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN7" s="1">
         <v>2.1682867107780601</v>
@@ -3691,17 +3695,17 @@
       <c r="AI10" s="1">
         <v>3.4375773834368202</v>
       </c>
-      <c r="AJ10" s="1">
-        <v>2.47573633254747E-2</v>
-      </c>
-      <c r="AK10" s="1">
-        <v>3.9430343603135E-2</v>
-      </c>
-      <c r="AL10" s="1">
-        <v>3.9333909745670297E-2</v>
-      </c>
-      <c r="AM10" s="1">
-        <v>0.62864471236902897</v>
+      <c r="AJ10" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK10" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL10" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM10" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN10" s="1">
         <v>9.6380702798517195</v>
@@ -4277,29 +4281,29 @@
       <c r="AE12" s="1">
         <v>10.385567058358101</v>
       </c>
-      <c r="AF12" s="1">
-        <v>3.5627610408862899E-2</v>
-      </c>
-      <c r="AG12" s="1">
-        <v>4.1955291521747998E-2</v>
-      </c>
-      <c r="AH12" s="1">
-        <v>4.1861358307647999E-2</v>
-      </c>
-      <c r="AI12" s="1">
-        <v>0.85013210759213598</v>
-      </c>
-      <c r="AJ12" s="1">
-        <v>5.5581437107919199E-2</v>
-      </c>
-      <c r="AK12" s="1">
-        <v>4.04461876713961E-2</v>
-      </c>
-      <c r="AL12" s="1">
-        <v>4.04610568941106E-2</v>
-      </c>
-      <c r="AM12" s="1">
-        <v>1.37395473381911</v>
+      <c r="AF12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM12" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN12" s="1">
         <v>30.187213114062299</v>
@@ -4558,17 +4562,17 @@
       <c r="Y13" s="1">
         <v>5.3401845970360897</v>
       </c>
-      <c r="Z13" s="1">
-        <v>3.9033681850017599E-2</v>
-      </c>
-      <c r="AA13" s="1">
-        <v>2.9207767290307701E-2</v>
-      </c>
-      <c r="AB13" s="1">
-        <v>2.9195231155963602E-2</v>
-      </c>
-      <c r="AC13" s="1">
-        <v>1.3367015228110399</v>
+      <c r="Z13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC13" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AD13" s="1">
         <v>6.6900579074547399E-3</v>
@@ -4576,29 +4580,29 @@
       <c r="AE13" s="1">
         <v>0.24446938514144101</v>
       </c>
-      <c r="AF13" s="1">
-        <v>6.0744815685438901E-2</v>
-      </c>
-      <c r="AG13" s="1">
-        <v>2.85063648909059E-2</v>
-      </c>
-      <c r="AH13" s="1">
-        <v>2.8528646203351899E-2</v>
-      </c>
-      <c r="AI13" s="1">
-        <v>2.1300895694266999</v>
-      </c>
-      <c r="AJ13" s="1">
-        <v>5.68097546442934E-3</v>
-      </c>
-      <c r="AK13" s="1">
-        <v>2.68998636624211E-2</v>
-      </c>
-      <c r="AL13" s="1">
-        <v>2.68069648108618E-2</v>
-      </c>
-      <c r="AM13" s="1">
-        <v>0.211555053575254</v>
+      <c r="AF13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM13" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN13" s="1">
         <v>7.0466332522027599</v>
@@ -5064,8 +5068,8 @@
       <c r="CP14" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="CQ14" s="4">
-        <v>0.71766908678116803</v>
+      <c r="CQ14" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="CR14" s="1">
         <v>12.4556042721387</v>
@@ -5096,17 +5100,17 @@
       <c r="E15" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="5">
-        <v>3261201.1723690098</v>
-      </c>
-      <c r="G15" s="5">
-        <v>6952277.5459529497</v>
-      </c>
-      <c r="H15" s="5">
-        <v>6922798.1831263499</v>
-      </c>
-      <c r="I15" s="5">
-        <v>0.47021429105448898</v>
+      <c r="F15" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="J15" s="1">
         <v>0.91296181444382896</v>
@@ -5156,17 +5160,17 @@
       <c r="Y15" s="1">
         <v>4.1547617654468096</v>
       </c>
-      <c r="Z15" s="1">
-        <v>1.7025933590205801E-2</v>
-      </c>
-      <c r="AA15" s="1">
-        <v>3.3644672103658298E-2</v>
-      </c>
-      <c r="AB15" s="1">
-        <v>3.3529773843771801E-2</v>
-      </c>
-      <c r="AC15" s="1">
-        <v>0.50691700228506398</v>
+      <c r="Z15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC15" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AD15" s="1">
         <v>8.4008435942035994E-3</v>
@@ -5174,29 +5178,29 @@
       <c r="AE15" s="1">
         <v>0.266690799862499</v>
       </c>
-      <c r="AF15" s="1">
-        <v>2.2548614646398801E-2</v>
-      </c>
-      <c r="AG15" s="1">
-        <v>3.1436923178959103E-2</v>
-      </c>
-      <c r="AH15" s="1">
-        <v>3.1407777458743402E-2</v>
-      </c>
-      <c r="AI15" s="1">
-        <v>0.71759803020630797</v>
-      </c>
-      <c r="AJ15" s="1">
-        <v>3.7792332212968897E-2</v>
-      </c>
-      <c r="AK15" s="1">
-        <v>3.2000321880836097E-2</v>
-      </c>
-      <c r="AL15" s="1">
-        <v>3.2000182501317601E-2</v>
-      </c>
-      <c r="AM15" s="1">
-        <v>1.1810013599616001</v>
+      <c r="AF15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM15" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN15" s="1">
         <v>3.4755646141877699</v>
@@ -6382,17 +6386,17 @@
       <c r="AI19" s="1">
         <v>3.0051120051273501</v>
       </c>
-      <c r="AJ19" s="1">
-        <v>6.40793379745698E-2</v>
-      </c>
-      <c r="AK19" s="1">
-        <v>2.6864837700766201E-2</v>
-      </c>
-      <c r="AL19" s="1">
-        <v>2.6864688222861598E-2</v>
-      </c>
-      <c r="AM19" s="1">
-        <v>2.3852574503511499</v>
+      <c r="AJ19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM19" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN19" s="1">
         <v>14.6538236901555</v>
@@ -7225,17 +7229,17 @@
       <c r="Q22" s="1">
         <v>41.629462222457597</v>
       </c>
-      <c r="R22" s="2">
-        <v>3.7522120129415401E-2</v>
-      </c>
-      <c r="S22" s="2">
-        <v>0.133765550322441</v>
-      </c>
-      <c r="T22" s="2">
-        <v>0.13315388895491301</v>
-      </c>
-      <c r="U22" s="2">
-        <v>0.28114940549546003</v>
+      <c r="R22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U22" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V22" s="1">
         <v>1.55314020044324</v>
@@ -7267,29 +7271,29 @@
       <c r="AE22" s="1">
         <v>8.2426119638353796</v>
       </c>
-      <c r="AF22" s="1">
-        <v>9.3473068333428805E-2</v>
-      </c>
-      <c r="AG22" s="1">
-        <v>0.108365059396476</v>
-      </c>
-      <c r="AH22" s="1">
-        <v>0.108082027991684</v>
-      </c>
-      <c r="AI22" s="1">
-        <v>0.86370376317137298</v>
-      </c>
-      <c r="AJ22" s="1">
-        <v>0.137112013375039</v>
-      </c>
-      <c r="AK22" s="1">
-        <v>0.105158683506754</v>
-      </c>
-      <c r="AL22" s="1">
-        <v>0.104846625724229</v>
-      </c>
-      <c r="AM22" s="1">
-        <v>1.3057961135407301</v>
+      <c r="AF22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM22" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN22" s="1">
         <v>27.210845331694301</v>
@@ -7566,29 +7570,29 @@
       <c r="AE23" s="1">
         <v>8.4093977156813899</v>
       </c>
-      <c r="AF23" s="1">
-        <v>1.07753450430492E-2</v>
-      </c>
-      <c r="AG23" s="1">
-        <v>3.9282868585672703E-2</v>
-      </c>
-      <c r="AH23" s="1">
-        <v>3.9051460986610803E-2</v>
-      </c>
-      <c r="AI23" s="1">
-        <v>0.27511169446058698</v>
-      </c>
-      <c r="AJ23" s="1">
-        <v>0.105583871120234</v>
-      </c>
-      <c r="AK23" s="1">
-        <v>3.8888676197133903E-2</v>
-      </c>
-      <c r="AL23" s="1">
-        <v>3.8824270868414099E-2</v>
-      </c>
-      <c r="AM23" s="1">
-        <v>2.7172794727267902</v>
+      <c r="AF23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM23" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN23" s="1">
         <v>18.062323514550101</v>
@@ -7877,17 +7881,17 @@
       <c r="AI24" s="1">
         <v>4.8104017252215998</v>
       </c>
-      <c r="AJ24" s="1">
-        <v>7.4604819648051199E-2</v>
-      </c>
-      <c r="AK24" s="1">
-        <v>5.1523430851219798E-2</v>
-      </c>
-      <c r="AL24" s="1">
-        <v>5.1532709155853097E-2</v>
-      </c>
-      <c r="AM24" s="1">
-        <v>1.4478481735772399</v>
+      <c r="AJ24" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK24" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL24" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM24" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN24" s="1">
         <v>77.713787597598497</v>
@@ -8463,29 +8467,29 @@
       <c r="AE26" s="1">
         <v>7.5148025542226096</v>
       </c>
-      <c r="AF26" s="1">
-        <v>5.2493958676664502E-2</v>
-      </c>
-      <c r="AG26" s="1">
-        <v>2.73702117129908E-2</v>
-      </c>
-      <c r="AH26" s="1">
-        <v>2.7312655340924499E-2</v>
-      </c>
-      <c r="AI26" s="1">
-        <v>1.9199421431585899</v>
-      </c>
-      <c r="AJ26" s="1">
-        <v>1.5781117974506102E-2</v>
-      </c>
-      <c r="AK26" s="1">
-        <v>2.45752574900618E-2</v>
-      </c>
-      <c r="AL26" s="1">
-        <v>2.45007473846694E-2</v>
-      </c>
-      <c r="AM26" s="1">
-        <v>0.64312970897636701</v>
+      <c r="AF26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM26" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN26" s="1">
         <v>11.4658426038771</v>
@@ -8720,17 +8724,17 @@
       <c r="Q27" s="1">
         <v>27.649913322798302</v>
       </c>
-      <c r="R27" s="2">
-        <v>0.215687743329776</v>
-      </c>
-      <c r="S27" s="2">
-        <v>9.4682190274357994E-2</v>
-      </c>
-      <c r="T27" s="2">
-        <v>9.4744615559859094E-2</v>
-      </c>
-      <c r="U27" s="2">
-        <v>2.2772714910297198</v>
+      <c r="R27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U27" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V27" s="1">
         <v>0.27897115865601502</v>
@@ -8846,17 +8850,17 @@
       <c r="BG27" s="1">
         <v>19.4042094943526</v>
       </c>
-      <c r="BH27" s="4">
-        <v>8.8428877078181395E-2</v>
-      </c>
-      <c r="BI27" s="4">
-        <v>3.5931074668569998E-2</v>
-      </c>
-      <c r="BJ27" s="4">
-        <v>3.5931074668569998E-2</v>
-      </c>
-      <c r="BK27" s="4">
-        <v>2.4552569820780299</v>
+      <c r="BH27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BI27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BJ27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BK27" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="BL27" s="1">
         <v>31.974868957351301</v>
@@ -9671,17 +9675,17 @@
       <c r="AI30" s="1">
         <v>3.8229008532126101</v>
       </c>
-      <c r="AJ30" s="1">
-        <v>0.31057572629763902</v>
-      </c>
-      <c r="AK30" s="1">
-        <v>0.108340340700719</v>
-      </c>
-      <c r="AL30" s="1">
-        <v>0.10839020331386801</v>
-      </c>
-      <c r="AM30" s="1">
-        <v>2.8660085109512399</v>
+      <c r="AJ30" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK30" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL30" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM30" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN30" s="1">
         <v>107.59271735893699</v>
@@ -11710,17 +11714,17 @@
       <c r="Q37" s="1">
         <v>38.107208653494901</v>
       </c>
-      <c r="R37" s="2">
-        <v>0.41985082353373299</v>
-      </c>
-      <c r="S37" s="2">
-        <v>0.15481043391286001</v>
-      </c>
-      <c r="T37" s="2">
-        <v>0.15456864828195799</v>
-      </c>
-      <c r="U37" s="2">
-        <v>2.7141559355843099</v>
+      <c r="R37" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S37" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T37" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U37" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V37" s="1">
         <v>1.0453428271757299</v>
@@ -11752,29 +11756,29 @@
       <c r="AE37" s="1">
         <v>4.9534557406544497</v>
       </c>
-      <c r="AF37" s="1">
-        <v>0.29096701621974502</v>
-      </c>
-      <c r="AG37" s="1">
-        <v>0.11939516949331699</v>
-      </c>
-      <c r="AH37" s="1">
-        <v>0.11960690985964301</v>
-      </c>
-      <c r="AI37" s="1">
-        <v>2.4348519792549599</v>
-      </c>
-      <c r="AJ37" s="1">
-        <v>0.129259663317985</v>
-      </c>
-      <c r="AK37" s="1">
-        <v>0.114487750145687</v>
-      </c>
-      <c r="AL37" s="1">
-        <v>0.11477550634155299</v>
-      </c>
-      <c r="AM37" s="1">
-        <v>1.1276093337836599</v>
+      <c r="AF37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM37" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN37" s="1">
         <v>27.452376893496201</v>
@@ -12350,17 +12354,17 @@
       <c r="AE39" s="1">
         <v>5.5112111335933998</v>
       </c>
-      <c r="AF39" s="1">
-        <v>2.5679764331849299E-2</v>
-      </c>
-      <c r="AG39" s="1">
-        <v>4.5370530966871499E-2</v>
-      </c>
-      <c r="AH39" s="1">
-        <v>4.5158661836185297E-2</v>
-      </c>
-      <c r="AI39" s="1">
-        <v>0.56732566408229501</v>
+      <c r="AF39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI39" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AJ39" s="1" t="s">
         <v>95</v>
@@ -12930,17 +12934,17 @@
       <c r="Y41" s="1">
         <v>2.9446572230624102</v>
       </c>
-      <c r="Z41" s="1">
-        <v>2.2487997330017499E-2</v>
-      </c>
-      <c r="AA41" s="1">
-        <v>2.9822094914211599E-2</v>
-      </c>
-      <c r="AB41" s="1">
-        <v>2.97457293923763E-2</v>
-      </c>
-      <c r="AC41" s="1">
-        <v>0.75503843649983304</v>
+      <c r="Z41" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA41" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB41" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC41" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AD41" s="1">
         <v>3.9473746993906697E-2</v>
@@ -13504,17 +13508,17 @@
       <c r="Q43" s="1">
         <v>26.603688006674599</v>
       </c>
-      <c r="R43" s="2">
-        <v>0.19558721703235099</v>
-      </c>
-      <c r="S43" s="2">
-        <v>0.104472271861867</v>
-      </c>
-      <c r="T43" s="2">
-        <v>0.104763822475557</v>
-      </c>
-      <c r="U43" s="2">
-        <v>1.8695412717030999</v>
+      <c r="R43" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S43" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T43" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U43" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V43" s="1">
         <v>0.87599768874086903</v>
@@ -13546,29 +13550,29 @@
       <c r="AE43" s="1">
         <v>5.4213192744580398</v>
       </c>
-      <c r="AF43" s="1">
-        <v>0.174382591855825</v>
-      </c>
-      <c r="AG43" s="1">
-        <v>8.3470604331970705E-2</v>
-      </c>
-      <c r="AH43" s="1">
-        <v>8.3187332599890598E-2</v>
-      </c>
-      <c r="AI43" s="1">
-        <v>2.0927066656235702</v>
-      </c>
-      <c r="AJ43" s="1">
-        <v>0.129095218172293</v>
-      </c>
-      <c r="AK43" s="1">
-        <v>7.8274208751807697E-2</v>
-      </c>
-      <c r="AL43" s="1">
-        <v>7.8341993434362295E-2</v>
-      </c>
-      <c r="AM43" s="1">
-        <v>1.6485579467875999</v>
+      <c r="AF43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM43" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN43" s="1">
         <v>16.752348920851801</v>
@@ -13803,17 +13807,17 @@
       <c r="Q44" s="1">
         <v>29.096161535016101</v>
       </c>
-      <c r="R44" s="2">
-        <v>0.41347809891817899</v>
-      </c>
-      <c r="S44" s="2">
-        <v>0.171551199791107</v>
-      </c>
-      <c r="T44" s="2">
-        <v>0.17132788314848901</v>
-      </c>
-      <c r="U44" s="2">
-        <v>2.41180699867631</v>
+      <c r="R44" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S44" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T44" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U44" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V44" s="1">
         <v>0.82183924106759498</v>
@@ -13857,17 +13861,17 @@
       <c r="AI44" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AJ44" s="1">
-        <v>0.30469152549532602</v>
-      </c>
-      <c r="AK44" s="1">
-        <v>0.12703491512842399</v>
-      </c>
-      <c r="AL44" s="1">
-        <v>0.127321180654625</v>
-      </c>
-      <c r="AM44" s="1">
-        <v>2.3957916575737599</v>
+      <c r="AJ44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM44" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN44" s="1">
         <v>28.1841266528583</v>
@@ -14106,7 +14110,7 @@
         <v>5.3512457655579597</v>
       </c>
       <c r="S45" s="2">
-        <v>1.3882839179236699E-2</v>
+        <v>1.3882838999999999E-2</v>
       </c>
       <c r="T45" s="2">
         <v>1.38972379807543E-2</v>
@@ -14401,17 +14405,17 @@
       <c r="Q46" s="1">
         <v>37.7728280801986</v>
       </c>
-      <c r="R46" s="2">
-        <v>0.27140486905400502</v>
-      </c>
-      <c r="S46" s="2">
-        <v>0.14899796978865301</v>
-      </c>
-      <c r="T46" s="2">
-        <v>0.14905445155779401</v>
-      </c>
-      <c r="U46" s="2">
-        <v>1.8211905021172401</v>
+      <c r="R46" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="S46" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T46" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="U46" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="V46" s="1">
         <v>1.3273315176801901</v>
@@ -14443,29 +14447,29 @@
       <c r="AE46" s="1">
         <v>6.4605205608724496</v>
       </c>
-      <c r="AF46" s="1">
-        <v>0.33770506134206002</v>
-      </c>
-      <c r="AG46" s="1">
-        <v>0.124365492021018</v>
-      </c>
-      <c r="AH46" s="1">
-        <v>0.12467648782308501</v>
-      </c>
-      <c r="AI46" s="1">
-        <v>2.7120377824194999</v>
-      </c>
-      <c r="AJ46" s="1">
-        <v>0.33501765648879001</v>
-      </c>
-      <c r="AK46" s="1">
-        <v>0.121246207986879</v>
-      </c>
-      <c r="AL46" s="1">
-        <v>0.12101084719269101</v>
-      </c>
-      <c r="AM46" s="1">
-        <v>2.7658078561902202</v>
+      <c r="AF46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AJ46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AM46" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="AN46" s="1">
         <v>28.901388479601898</v>

</xml_diff>